<commit_message>
Add PSF data visualisation
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -1,27 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80B8953C-7C49-B14F-9ABB-C03BDF22251D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC00ED9-9634-2746-905F-5B268F7B1F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="60160" windowHeight="31920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25680" windowHeight="20940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="laser_power_objective_measureme" sheetId="1" r:id="rId1"/>
     <sheet name="psf_measurements" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="38">
   <si>
     <t>Site</t>
   </si>
@@ -114,6 +127,27 @@
   </si>
   <si>
     <t>Pinhole open</t>
+  </si>
+  <si>
+    <t>Mic1</t>
+  </si>
+  <si>
+    <t>Mic2</t>
+  </si>
+  <si>
+    <t>10x/1.1</t>
+  </si>
+  <si>
+    <t>Mic3</t>
+  </si>
+  <si>
+    <t>Mic4</t>
+  </si>
+  <si>
+    <t>20100101-2</t>
+  </si>
+  <si>
+    <t>20200101something</t>
   </si>
 </sst>
 </file>
@@ -245,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -317,9 +351,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -3694,13 +3725,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3720,12 +3751,19 @@
         <v>19</v>
       </c>
       <c r="G1" s="31">
-        <v>20100101</v>
-      </c>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>20150101</v>
+      </c>
+      <c r="H1" s="31">
+        <v>20131212</v>
+      </c>
+      <c r="I1" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="J1" s="31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="32" t="s">
         <v>7</v>
       </c>
@@ -3747,9 +3785,17 @@
       <c r="G2" s="6">
         <v>200</v>
       </c>
-      <c r="H2" s="33"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H2" s="6"/>
+      <c r="I2" s="32">
+        <f>G2/2</f>
+        <v>100</v>
+      </c>
+      <c r="J2">
+        <f>G2*2</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="32" t="s">
         <v>7</v>
       </c>
@@ -3771,9 +3817,17 @@
       <c r="G3" s="6">
         <v>200</v>
       </c>
-      <c r="H3" s="33"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H3" s="6"/>
+      <c r="I3" s="32">
+        <f t="shared" ref="I3:I28" si="0">G3/2</f>
+        <v>100</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J28" si="1">G3*2</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="32" t="s">
         <v>7</v>
       </c>
@@ -3795,10 +3849,17 @@
       <c r="G4" s="6">
         <v>500</v>
       </c>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H4" s="6"/>
+      <c r="I4" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="32" t="s">
         <v>7</v>
       </c>
@@ -3820,9 +3881,17 @@
       <c r="G5" s="6">
         <v>200</v>
       </c>
-      <c r="I5" s="33"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H5" s="6"/>
+      <c r="I5" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="32" t="s">
         <v>7</v>
       </c>
@@ -3844,9 +3913,17 @@
       <c r="G6" s="6">
         <v>200</v>
       </c>
-      <c r="I6" s="33"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H6" s="6"/>
+      <c r="I6" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="32" t="s">
         <v>7</v>
       </c>
@@ -3868,9 +3945,17 @@
       <c r="G7" s="6">
         <v>500</v>
       </c>
-      <c r="I7" s="33"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H7" s="6"/>
+      <c r="I7" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="32" t="s">
         <v>7</v>
       </c>
@@ -3892,9 +3977,17 @@
       <c r="G8" s="6">
         <v>200</v>
       </c>
-      <c r="I8" s="33"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H8" s="6"/>
+      <c r="I8" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="32" t="s">
         <v>7</v>
       </c>
@@ -3916,9 +4009,17 @@
       <c r="G9" s="6">
         <v>200</v>
       </c>
-      <c r="I9" s="33"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H9" s="6"/>
+      <c r="I9" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="32" t="s">
         <v>7</v>
       </c>
@@ -3940,9 +4041,17 @@
       <c r="G10" s="6">
         <v>500</v>
       </c>
-      <c r="I10" s="33"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H10" s="6"/>
+      <c r="I10" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="32" t="s">
         <v>7</v>
       </c>
@@ -3964,8 +4073,17 @@
       <c r="G11" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H11" s="6"/>
+      <c r="I11" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="32" t="s">
         <v>7</v>
       </c>
@@ -3987,8 +4105,17 @@
       <c r="G12" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H12" s="6"/>
+      <c r="I12" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="32" t="s">
         <v>7</v>
       </c>
@@ -4010,10 +4137,19 @@
       <c r="G13" s="6">
         <v>500</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H13" s="6"/>
+      <c r="I13" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B14" s="32" t="s">
         <v>20</v>
@@ -4033,10 +4169,21 @@
       <c r="G14" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H14" s="6">
+        <v>200</v>
+      </c>
+      <c r="I14" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B15" s="32" t="s">
         <v>20</v>
@@ -4056,10 +4203,21 @@
       <c r="G15" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H15" s="6">
+        <v>200</v>
+      </c>
+      <c r="I15" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B16" s="32" t="s">
         <v>20</v>
@@ -4079,10 +4237,21 @@
       <c r="G16" s="6">
         <v>500</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H16" s="6">
+        <v>500</v>
+      </c>
+      <c r="I16" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B17" s="32" t="s">
         <v>20</v>
@@ -4102,10 +4271,21 @@
       <c r="G17" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H17" s="6">
+        <v>200</v>
+      </c>
+      <c r="I17" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B18" s="32" t="s">
         <v>20</v>
@@ -4125,10 +4305,21 @@
       <c r="G18" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H18" s="6">
+        <v>200</v>
+      </c>
+      <c r="I18" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B19" s="32" t="s">
         <v>20</v>
@@ -4148,10 +4339,21 @@
       <c r="G19" s="6">
         <v>500</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H19" s="6">
+        <v>500</v>
+      </c>
+      <c r="I19" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B20" s="32" t="s">
         <v>20</v>
@@ -4171,10 +4373,21 @@
       <c r="G20" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H20" s="6">
+        <v>200</v>
+      </c>
+      <c r="I20" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B21" s="32" t="s">
         <v>20</v>
@@ -4194,10 +4407,21 @@
       <c r="G21" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H21" s="6">
+        <v>200</v>
+      </c>
+      <c r="I21" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B22" s="32" t="s">
         <v>20</v>
@@ -4217,10 +4441,21 @@
       <c r="G22" s="6">
         <v>500</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H22" s="6">
+        <v>500</v>
+      </c>
+      <c r="I22" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B23" s="32" t="s">
         <v>20</v>
@@ -4240,10 +4475,21 @@
       <c r="G23" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H23" s="6">
+        <v>200</v>
+      </c>
+      <c r="I23" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B24" s="32" t="s">
         <v>20</v>
@@ -4263,13 +4509,24 @@
       <c r="G24" s="6">
         <v>200</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H24" s="6">
+        <v>200</v>
+      </c>
+      <c r="I24" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="32" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B25" s="32" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C25" s="32" t="s">
         <v>21</v>
@@ -4286,35 +4543,113 @@
       <c r="G25" s="6">
         <v>500</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="32"/>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="6"/>
-    </row>
-    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="32"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="6"/>
-    </row>
-    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="32"/>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="6"/>
-    </row>
-    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H25" s="6"/>
+      <c r="I25" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F26" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="6">
+        <v>500</v>
+      </c>
+      <c r="H26" s="6"/>
+      <c r="I26" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A27" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="D27" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="6">
+        <v>500</v>
+      </c>
+      <c r="H27" s="6"/>
+      <c r="I27" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="6">
+        <v>500</v>
+      </c>
+      <c r="H28" s="6"/>
+      <c r="I28" s="32">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="32"/>
       <c r="B29" s="32"/>
       <c r="C29" s="32"/>
@@ -4322,8 +4657,9 @@
       <c r="E29" s="32"/>
       <c r="F29" s="32"/>
       <c r="G29" s="6"/>
-    </row>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H29" s="6"/>
+    </row>
+    <row r="30" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="32"/>
       <c r="B30" s="32"/>
       <c r="C30" s="32"/>
@@ -4331,8 +4667,9 @@
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
       <c r="G30" s="6"/>
-    </row>
-    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H30" s="6"/>
+    </row>
+    <row r="31" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="32"/>
       <c r="B31" s="32"/>
       <c r="C31" s="32"/>
@@ -4340,8 +4677,9 @@
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
       <c r="G31" s="6"/>
-    </row>
-    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H31" s="6"/>
+    </row>
+    <row r="32" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="32"/>
       <c r="B32" s="32"/>
       <c r="C32" s="32"/>
@@ -4349,8 +4687,9 @@
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
       <c r="G32" s="6"/>
-    </row>
-    <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H32" s="6"/>
+    </row>
+    <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="32"/>
       <c r="B33" s="32"/>
       <c r="C33" s="32"/>
@@ -4358,8 +4697,9 @@
       <c r="E33" s="32"/>
       <c r="F33" s="32"/>
       <c r="G33" s="6"/>
-    </row>
-    <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H33" s="6"/>
+    </row>
+    <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="32"/>
       <c r="B34" s="32"/>
       <c r="C34" s="32"/>
@@ -4367,8 +4707,9 @@
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
       <c r="G34" s="6"/>
-    </row>
-    <row r="35" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H34" s="6"/>
+    </row>
+    <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="32"/>
       <c r="B35" s="32"/>
       <c r="C35" s="32"/>
@@ -4376,8 +4717,9 @@
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
       <c r="G35" s="6"/>
-    </row>
-    <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H35" s="6"/>
+    </row>
+    <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="32"/>
       <c r="B36" s="32"/>
       <c r="C36" s="32"/>
@@ -4385,8 +4727,9 @@
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
       <c r="G36" s="6"/>
-    </row>
-    <row r="37" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="H36" s="6"/>
+    </row>
+    <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="32"/>
       <c r="B37" s="32"/>
       <c r="C37" s="32"/>
@@ -4394,6 +4737,7 @@
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
       <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Rewrite power app & change sheet names (breaking)
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC00ED9-9634-2746-905F-5B268F7B1F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9075D07-02C6-F74A-AAB4-97AF5F1C4E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25680" windowHeight="20940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="laser_power_objective_measureme" sheetId="1" r:id="rId1"/>
+    <sheet name="laser_power_measurements" sheetId="1" r:id="rId1"/>
     <sheet name="psf_measurements" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="41">
   <si>
     <t>Site</t>
   </si>
@@ -148,6 +148,15 @@
   </si>
   <si>
     <t>20200101something</t>
+  </si>
+  <si>
+    <t>20190910text</t>
+  </si>
+  <si>
+    <t>20150101-sort</t>
+  </si>
+  <si>
+    <t>no_data</t>
   </si>
 </sst>
 </file>
@@ -279,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -353,6 +362,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,7 +585,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:BZ46"/>
+  <dimension ref="A1:BZ47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="26" max="26" width="13.1640625" customWidth="1"/>
@@ -604,13 +614,15 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2">
-        <v>20190910</v>
+      <c r="H1" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="I1" s="2">
         <v>20191008</v>
       </c>
-      <c r="J1" s="2"/>
+      <c r="J1" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
@@ -702,10 +714,12 @@
       <c r="H2" s="8">
         <v>8.2899999999999991</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="8">
         <v>7.63</v>
       </c>
-      <c r="J2" s="8"/>
+      <c r="J2" s="8">
+        <v>7.63</v>
+      </c>
       <c r="K2" s="8"/>
       <c r="L2" s="10"/>
       <c r="M2" s="8"/>
@@ -775,10 +789,12 @@
       <c r="H3" s="8">
         <v>16.600000000000001</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="8">
         <v>15.8</v>
       </c>
-      <c r="J3" s="8"/>
+      <c r="J3" s="8">
+        <v>15.8</v>
+      </c>
       <c r="K3" s="8"/>
       <c r="L3" s="10"/>
       <c r="M3" s="8"/>
@@ -848,10 +864,12 @@
       <c r="H4" s="8">
         <v>81.5</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="8">
         <v>79.5</v>
       </c>
-      <c r="J4" s="8"/>
+      <c r="J4" s="8">
+        <v>79.5</v>
+      </c>
       <c r="K4" s="8"/>
       <c r="L4" s="10"/>
       <c r="M4" s="8"/>
@@ -921,10 +939,12 @@
       <c r="H5" s="8">
         <v>146</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="8">
         <v>143</v>
       </c>
-      <c r="J5" s="8"/>
+      <c r="J5" s="8">
+        <v>143</v>
+      </c>
       <c r="K5" s="8"/>
       <c r="L5" s="10"/>
       <c r="M5" s="8"/>
@@ -994,10 +1014,12 @@
       <c r="H6" s="8">
         <v>162</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="8">
         <v>159</v>
       </c>
-      <c r="J6" s="8"/>
+      <c r="J6" s="8">
+        <v>159</v>
+      </c>
       <c r="K6" s="8"/>
       <c r="L6" s="16"/>
       <c r="M6" s="8"/>
@@ -1067,10 +1089,12 @@
       <c r="H7" s="8">
         <v>12.5</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="8">
         <v>10.5</v>
       </c>
-      <c r="J7" s="8"/>
+      <c r="J7" s="8">
+        <v>10.5</v>
+      </c>
       <c r="K7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
@@ -1139,10 +1163,12 @@
       <c r="H8" s="8">
         <v>24.5</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="8">
         <v>22.5</v>
       </c>
-      <c r="J8" s="8"/>
+      <c r="J8" s="8">
+        <v>22.5</v>
+      </c>
       <c r="K8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
@@ -1211,10 +1237,12 @@
       <c r="H9" s="8">
         <v>122</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="8">
         <v>119</v>
       </c>
-      <c r="J9" s="8"/>
+      <c r="J9" s="8">
+        <v>119</v>
+      </c>
       <c r="K9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
@@ -1283,10 +1311,12 @@
       <c r="H10" s="8">
         <v>218</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="8">
         <v>215</v>
       </c>
-      <c r="J10" s="8"/>
+      <c r="J10" s="8">
+        <v>215</v>
+      </c>
       <c r="K10" s="8"/>
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
@@ -1355,10 +1385,12 @@
       <c r="H11" s="8">
         <v>242</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="8">
         <v>239</v>
       </c>
-      <c r="J11" s="8"/>
+      <c r="J11" s="8">
+        <v>239</v>
+      </c>
       <c r="K11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
@@ -1427,10 +1459,12 @@
       <c r="H12" s="8">
         <v>11.1</v>
       </c>
-      <c r="I12" s="11">
+      <c r="I12" s="8">
         <v>10.7</v>
       </c>
-      <c r="J12" s="8"/>
+      <c r="J12" s="8">
+        <v>10.7</v>
+      </c>
       <c r="K12" s="8"/>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
@@ -1499,10 +1533,12 @@
       <c r="H13" s="8">
         <v>22.7</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="8">
         <v>22.2</v>
       </c>
-      <c r="J13" s="8"/>
+      <c r="J13" s="8">
+        <v>22.2</v>
+      </c>
       <c r="K13" s="8"/>
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
@@ -1571,10 +1607,12 @@
       <c r="H14" s="8">
         <v>115</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="8">
         <v>115</v>
       </c>
-      <c r="J14" s="8"/>
+      <c r="J14" s="8">
+        <v>115</v>
+      </c>
       <c r="K14" s="8"/>
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
@@ -1643,10 +1681,12 @@
       <c r="H15" s="8">
         <v>210</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15" s="8">
         <v>209</v>
       </c>
-      <c r="J15" s="8"/>
+      <c r="J15" s="8">
+        <v>209</v>
+      </c>
       <c r="K15" s="8"/>
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
@@ -1715,10 +1755,12 @@
       <c r="H16" s="8">
         <v>234</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="8">
         <v>232</v>
       </c>
-      <c r="J16" s="8"/>
+      <c r="J16" s="8">
+        <v>232</v>
+      </c>
       <c r="K16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
@@ -1787,10 +1829,12 @@
       <c r="H17" s="8">
         <v>3.61</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="8">
         <v>3.13</v>
       </c>
-      <c r="J17" s="8"/>
+      <c r="J17" s="8">
+        <v>3.13</v>
+      </c>
       <c r="K17" s="8"/>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
@@ -1859,10 +1903,12 @@
       <c r="H18" s="8">
         <v>7.11</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18" s="8">
         <v>6.7</v>
       </c>
-      <c r="J18" s="8"/>
+      <c r="J18" s="8">
+        <v>6.7</v>
+      </c>
       <c r="K18" s="8"/>
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
@@ -1931,10 +1977,12 @@
       <c r="H19" s="8">
         <v>36.299999999999997</v>
       </c>
-      <c r="I19" s="9">
+      <c r="I19" s="8">
         <v>34.6</v>
       </c>
-      <c r="J19" s="8"/>
+      <c r="J19" s="8">
+        <v>34.6</v>
+      </c>
       <c r="K19" s="8"/>
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
@@ -2003,10 +2051,12 @@
       <c r="H20" s="8">
         <v>63.4</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20" s="8">
         <v>61.6</v>
       </c>
-      <c r="J20" s="8"/>
+      <c r="J20" s="8">
+        <v>61.6</v>
+      </c>
       <c r="K20" s="8"/>
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
@@ -2075,10 +2125,12 @@
       <c r="H21" s="8">
         <v>69.7</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="8">
         <v>67.7</v>
       </c>
-      <c r="J21" s="8"/>
+      <c r="J21" s="8">
+        <v>67.7</v>
+      </c>
       <c r="K21" s="8"/>
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
@@ -2147,10 +2199,12 @@
       <c r="H22" s="8">
         <v>2.41</v>
       </c>
-      <c r="I22" s="22">
+      <c r="I22" s="8">
         <v>2.0299999999999998</v>
       </c>
-      <c r="J22" s="8"/>
+      <c r="J22" s="8">
+        <v>2.0299999999999998</v>
+      </c>
       <c r="K22" s="8"/>
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
@@ -2219,10 +2273,12 @@
       <c r="H23" s="8">
         <v>4.9400000000000004</v>
       </c>
-      <c r="I23" s="9">
+      <c r="I23" s="8">
         <v>4.66</v>
       </c>
-      <c r="J23" s="8"/>
+      <c r="J23" s="8">
+        <v>4.66</v>
+      </c>
       <c r="K23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
@@ -2291,10 +2347,12 @@
       <c r="H24" s="8">
         <v>24.3</v>
       </c>
-      <c r="I24" s="11">
+      <c r="I24" s="8">
         <v>23.8</v>
       </c>
-      <c r="J24" s="8"/>
+      <c r="J24" s="8">
+        <v>23.8</v>
+      </c>
       <c r="K24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
@@ -2363,10 +2421,12 @@
       <c r="H25" s="8">
         <v>43.4</v>
       </c>
-      <c r="I25" s="9">
+      <c r="I25" s="8">
         <v>43.1</v>
       </c>
-      <c r="J25" s="8"/>
+      <c r="J25" s="8">
+        <v>43.1</v>
+      </c>
       <c r="K25" s="8"/>
       <c r="M25" s="8"/>
       <c r="N25" s="8"/>
@@ -2435,10 +2495,12 @@
       <c r="H26" s="8">
         <v>48.1</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26" s="8">
         <v>47.2</v>
       </c>
-      <c r="J26" s="8"/>
+      <c r="J26" s="8">
+        <v>47.2</v>
+      </c>
       <c r="K26" s="8"/>
       <c r="M26" s="8"/>
       <c r="N26" s="8"/>
@@ -2504,13 +2566,15 @@
       <c r="G27" s="7">
         <v>5</v>
       </c>
-      <c r="H27" s="26">
+      <c r="H27" s="8">
         <v>0.157</v>
       </c>
-      <c r="I27" s="26">
+      <c r="I27" s="8">
         <v>0.17100000000000001</v>
       </c>
-      <c r="J27" s="26"/>
+      <c r="J27" s="8">
+        <v>0.17100000000000001</v>
+      </c>
       <c r="K27" s="26"/>
       <c r="M27" s="9"/>
       <c r="N27" s="27"/>
@@ -2567,13 +2631,15 @@
       <c r="G28" s="7">
         <v>10</v>
       </c>
-      <c r="H28" s="26">
+      <c r="H28" s="8">
         <v>0.308</v>
       </c>
-      <c r="I28" s="26">
+      <c r="I28" s="8">
         <v>0.34</v>
       </c>
-      <c r="J28" s="26"/>
+      <c r="J28" s="8">
+        <v>0.34</v>
+      </c>
       <c r="K28" s="26"/>
       <c r="M28" s="9"/>
       <c r="N28" s="27"/>
@@ -2630,13 +2696,15 @@
       <c r="G29" s="7">
         <v>50</v>
       </c>
-      <c r="H29" s="9">
+      <c r="H29" s="8">
         <v>1.45</v>
       </c>
-      <c r="I29" s="9">
+      <c r="I29" s="8">
         <v>1.62</v>
       </c>
-      <c r="J29" s="27"/>
+      <c r="J29" s="8">
+        <v>1.62</v>
+      </c>
       <c r="K29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="27"/>
@@ -2693,13 +2761,15 @@
       <c r="G30" s="7">
         <v>90</v>
       </c>
-      <c r="H30" s="9">
+      <c r="H30" s="8">
         <v>2.5299999999999998</v>
       </c>
-      <c r="I30" s="9">
+      <c r="I30" s="8">
         <v>2.87</v>
       </c>
-      <c r="J30" s="11"/>
+      <c r="J30" s="8">
+        <v>2.87</v>
+      </c>
       <c r="K30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9"/>
@@ -2756,13 +2826,15 @@
       <c r="G31" s="7">
         <v>100</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31" s="8">
         <v>2.78</v>
       </c>
-      <c r="I31" s="9">
+      <c r="I31" s="8">
         <v>3.17</v>
       </c>
-      <c r="J31" s="9"/>
+      <c r="J31" s="8">
+        <v>3.17</v>
+      </c>
       <c r="K31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9"/>
@@ -2819,13 +2891,15 @@
       <c r="G32" s="17">
         <v>5</v>
       </c>
-      <c r="H32" s="9">
+      <c r="H32" s="8">
         <v>0.46</v>
       </c>
-      <c r="I32" s="27">
+      <c r="I32" s="8">
         <v>0.46400000000000002</v>
       </c>
-      <c r="J32" s="9"/>
+      <c r="J32" s="8">
+        <v>0.46400000000000002</v>
+      </c>
       <c r="K32" s="27"/>
       <c r="M32" s="9"/>
       <c r="N32" s="27"/>
@@ -2882,13 +2956,15 @@
       <c r="G33" s="17">
         <v>10</v>
       </c>
-      <c r="H33" s="9">
+      <c r="H33" s="8">
         <v>0.89</v>
       </c>
-      <c r="I33" s="27">
+      <c r="I33" s="8">
         <v>0.89500000000000002</v>
       </c>
-      <c r="J33" s="27"/>
+      <c r="J33" s="8">
+        <v>0.89500000000000002</v>
+      </c>
       <c r="K33" s="27"/>
       <c r="M33" s="9"/>
       <c r="N33" s="27"/>
@@ -2945,13 +3021,15 @@
       <c r="G34" s="17">
         <v>50</v>
       </c>
-      <c r="H34" s="9">
+      <c r="H34" s="8">
         <v>4.26</v>
       </c>
-      <c r="I34" s="9">
+      <c r="I34" s="8">
         <v>4.26</v>
       </c>
-      <c r="J34" s="9"/>
+      <c r="J34" s="8">
+        <v>4.26</v>
+      </c>
       <c r="K34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9"/>
@@ -3008,13 +3086,15 @@
       <c r="G35" s="17">
         <v>90</v>
       </c>
-      <c r="H35" s="9">
+      <c r="H35" s="8">
         <v>7.46</v>
       </c>
-      <c r="I35" s="11">
+      <c r="I35" s="8">
         <v>7.5</v>
       </c>
-      <c r="J35" s="9"/>
+      <c r="J35" s="8">
+        <v>7.5</v>
+      </c>
       <c r="K35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
@@ -3071,13 +3151,15 @@
       <c r="G36" s="17">
         <v>100</v>
       </c>
-      <c r="H36" s="9">
+      <c r="H36" s="8">
         <v>8.17</v>
       </c>
-      <c r="I36" s="9">
+      <c r="I36" s="8">
         <v>8.23</v>
       </c>
-      <c r="J36" s="9"/>
+      <c r="J36" s="8">
+        <v>8.23</v>
+      </c>
       <c r="K36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9"/>
@@ -3134,13 +3216,15 @@
       <c r="G37" s="7">
         <v>5</v>
       </c>
-      <c r="H37" s="12" t="s">
+      <c r="H37" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="I37" s="9">
+      <c r="I37" s="8">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="J37" s="9"/>
+      <c r="J37" s="8">
+        <v>2.7000000000000001E-3</v>
+      </c>
       <c r="K37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9"/>
@@ -3194,13 +3278,15 @@
       <c r="G38" s="7">
         <v>10</v>
       </c>
-      <c r="H38" s="12" t="s">
+      <c r="H38" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="I38" s="9">
+      <c r="I38" s="8">
         <v>0.3</v>
       </c>
-      <c r="J38" s="9"/>
+      <c r="J38" s="8">
+        <v>0.3</v>
+      </c>
       <c r="K38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9"/>
@@ -3254,13 +3340,15 @@
       <c r="G39" s="7">
         <v>50</v>
       </c>
-      <c r="H39" s="12" t="s">
+      <c r="H39" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="I39" s="9">
+      <c r="I39" s="8">
         <v>6.17</v>
       </c>
-      <c r="J39" s="9"/>
+      <c r="J39" s="8">
+        <v>6.17</v>
+      </c>
       <c r="K39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9"/>
@@ -3314,13 +3402,15 @@
       <c r="G40" s="7">
         <v>90</v>
       </c>
-      <c r="H40" s="9">
+      <c r="H40" s="8">
         <v>10.199999999999999</v>
       </c>
-      <c r="I40" s="9">
+      <c r="I40" s="8">
         <v>10.8</v>
       </c>
-      <c r="J40" s="9"/>
+      <c r="J40" s="8">
+        <v>10.8</v>
+      </c>
       <c r="K40" s="9"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9"/>
@@ -3374,13 +3464,15 @@
       <c r="G41" s="7">
         <v>100</v>
       </c>
-      <c r="H41" s="9">
+      <c r="H41" s="8">
         <v>11</v>
       </c>
-      <c r="I41" s="9">
+      <c r="I41" s="8">
         <v>11.7</v>
       </c>
-      <c r="J41" s="9"/>
+      <c r="J41" s="8">
+        <v>11.7</v>
+      </c>
       <c r="K41" s="9"/>
       <c r="M41" s="9"/>
       <c r="N41" s="9"/>
@@ -3434,13 +3526,15 @@
       <c r="G42" s="17">
         <v>5</v>
       </c>
-      <c r="H42" s="9">
+      <c r="H42" s="8">
         <v>0.77200000000000002</v>
       </c>
-      <c r="I42" s="9">
+      <c r="I42" s="8">
         <v>0.83099999999999996</v>
       </c>
-      <c r="J42" s="9"/>
+      <c r="J42" s="8">
+        <v>0.83099999999999996</v>
+      </c>
       <c r="K42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9"/>
@@ -3494,13 +3588,15 @@
       <c r="G43" s="17">
         <v>10</v>
       </c>
-      <c r="H43" s="9">
+      <c r="H43" s="8">
         <v>1.42</v>
       </c>
-      <c r="I43" s="9">
+      <c r="I43" s="8">
         <v>1.54</v>
       </c>
-      <c r="J43" s="9"/>
+      <c r="J43" s="8">
+        <v>1.54</v>
+      </c>
       <c r="K43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9"/>
@@ -3554,13 +3650,15 @@
       <c r="G44" s="17">
         <v>50</v>
       </c>
-      <c r="H44" s="9">
+      <c r="H44" s="8">
         <v>5.4</v>
       </c>
-      <c r="I44" s="9">
+      <c r="I44" s="8">
         <v>5.81</v>
       </c>
-      <c r="J44" s="9"/>
+      <c r="J44" s="8">
+        <v>5.81</v>
+      </c>
       <c r="K44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
@@ -3614,13 +3712,15 @@
       <c r="G45" s="17">
         <v>90</v>
       </c>
-      <c r="H45" s="9">
+      <c r="H45" s="8">
         <v>7.82</v>
       </c>
-      <c r="I45" s="9">
+      <c r="I45" s="8">
         <v>8.51</v>
       </c>
-      <c r="J45" s="9"/>
+      <c r="J45" s="8">
+        <v>8.51</v>
+      </c>
       <c r="K45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9"/>
@@ -3674,13 +3774,15 @@
       <c r="G46" s="17">
         <v>100</v>
       </c>
-      <c r="H46" s="9">
+      <c r="H46" s="8">
         <v>8.25</v>
       </c>
-      <c r="I46" s="9">
+      <c r="I46" s="8">
         <v>9.0500000000000007</v>
       </c>
-      <c r="J46" s="9"/>
+      <c r="J46" s="8">
+        <v>9.0500000000000007</v>
+      </c>
       <c r="K46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9"/>
@@ -3715,6 +3817,26 @@
       <c r="BQ46" s="21"/>
       <c r="BS46" s="24"/>
     </row>
+    <row r="47" spans="1:75" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E47">
+        <v>561</v>
+      </c>
+      <c r="G47" s="17">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update PSF app: rewrite and shift plot
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9075D07-02C6-F74A-AAB4-97AF5F1C4E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F08F61-A961-E24A-8D60-D986712F5C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="laser_power_measurements" sheetId="1" r:id="rId1"/>
     <sheet name="psf_measurements" sheetId="2" r:id="rId2"/>
+    <sheet name="objective_db" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="93">
   <si>
     <t>Site</t>
   </si>
@@ -157,6 +158,162 @@
   </si>
   <si>
     <t>no_data</t>
+  </si>
+  <si>
+    <t>Test Entry</t>
+  </si>
+  <si>
+    <t>Shift-X</t>
+  </si>
+  <si>
+    <t>Shift-Y</t>
+  </si>
+  <si>
+    <t>Shift-Z</t>
+  </si>
+  <si>
+    <t>Reference-X</t>
+  </si>
+  <si>
+    <t>Reference-Y</t>
+  </si>
+  <si>
+    <t>Reference-Z</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Magnification</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Refractive Index</t>
+  </si>
+  <si>
+    <t>Working Distance [mm]</t>
+  </si>
+  <si>
+    <t>Ph</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Belongs to system</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>Vendor ID</t>
+  </si>
+  <si>
+    <t>Purchase date</t>
+  </si>
+  <si>
+    <t>ID1</t>
+  </si>
+  <si>
+    <t>CFI Plan Apo λ</t>
+  </si>
+  <si>
+    <t>4x</t>
+  </si>
+  <si>
+    <t>Air</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>on system</t>
+  </si>
+  <si>
+    <t>BSL2</t>
+  </si>
+  <si>
+    <t>Nikon</t>
+  </si>
+  <si>
+    <t>MRD00045</t>
+  </si>
+  <si>
+    <t>ID2</t>
+  </si>
+  <si>
+    <t>10x</t>
+  </si>
+  <si>
+    <t>MRD00105</t>
+  </si>
+  <si>
+    <t>ID3</t>
+  </si>
+  <si>
+    <t>20x</t>
+  </si>
+  <si>
+    <t>MRD00205</t>
+  </si>
+  <si>
+    <t>ID4</t>
+  </si>
+  <si>
+    <t>40x</t>
+  </si>
+  <si>
+    <t>0.25-0-17</t>
+  </si>
+  <si>
+    <t>MRD00405</t>
+  </si>
+  <si>
+    <t>ID5</t>
+  </si>
+  <si>
+    <t>100x</t>
+  </si>
+  <si>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>EXT Ph4</t>
+  </si>
+  <si>
+    <t>Ti2</t>
+  </si>
+  <si>
+    <t>MRD01905</t>
+  </si>
+  <si>
+    <t>ID19</t>
+  </si>
+  <si>
+    <t>60x</t>
+  </si>
+  <si>
+    <t>EXT Ph3</t>
+  </si>
+  <si>
+    <t>Cupboard</t>
+  </si>
+  <si>
+    <t>CSU-W1</t>
+  </si>
+  <si>
+    <t>MRD01605</t>
+  </si>
+  <si>
+    <t>cupboard</t>
   </si>
 </sst>
 </file>
@@ -168,7 +325,7 @@
     <numFmt numFmtId="165" formatCode="dd\.mm"/>
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -267,6 +424,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -288,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -363,6 +533,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,7 +763,7 @@
     <col min="30" max="31" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,7 +863,7 @@
       <c r="BY1" s="2"/>
       <c r="BZ1" s="2"/>
     </row>
-    <row r="2" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
@@ -767,7 +938,7 @@
       <c r="BY2" s="13"/>
       <c r="BZ2" s="13"/>
     </row>
-    <row r="3" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
@@ -842,7 +1013,7 @@
       <c r="BY3" s="13"/>
       <c r="BZ3" s="13"/>
     </row>
-    <row r="4" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
@@ -917,7 +1088,7 @@
       <c r="BY4" s="13"/>
       <c r="BZ4" s="13"/>
     </row>
-    <row r="5" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -992,7 +1163,7 @@
       <c r="BY5" s="15"/>
       <c r="BZ5" s="15"/>
     </row>
-    <row r="6" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -1067,7 +1238,7 @@
       <c r="BY6" s="15"/>
       <c r="BZ6" s="15"/>
     </row>
-    <row r="7" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -1141,7 +1312,7 @@
       <c r="BY7" s="19"/>
       <c r="BZ7" s="19"/>
     </row>
-    <row r="8" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -1215,7 +1386,7 @@
       <c r="BY8" s="19"/>
       <c r="BZ8" s="19"/>
     </row>
-    <row r="9" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -1289,7 +1460,7 @@
       <c r="BY9" s="15"/>
       <c r="BZ9" s="15"/>
     </row>
-    <row r="10" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -1363,7 +1534,7 @@
       <c r="BY10" s="15"/>
       <c r="BZ10" s="15"/>
     </row>
-    <row r="11" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -1437,7 +1608,7 @@
       <c r="BY11" s="15"/>
       <c r="BZ11" s="15"/>
     </row>
-    <row r="12" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>7</v>
       </c>
@@ -1511,7 +1682,7 @@
       <c r="BY12" s="19"/>
       <c r="BZ12" s="19"/>
     </row>
-    <row r="13" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>7</v>
       </c>
@@ -1585,7 +1756,7 @@
       <c r="BY13" s="19"/>
       <c r="BZ13" s="19"/>
     </row>
-    <row r="14" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
@@ -1659,7 +1830,7 @@
       <c r="BY14" s="15"/>
       <c r="BZ14" s="15"/>
     </row>
-    <row r="15" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>7</v>
       </c>
@@ -1733,7 +1904,7 @@
       <c r="BY15" s="15"/>
       <c r="BZ15" s="15"/>
     </row>
-    <row r="16" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>7</v>
       </c>
@@ -1807,7 +1978,7 @@
       <c r="BY16" s="15"/>
       <c r="BZ16" s="15"/>
     </row>
-    <row r="17" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>7</v>
       </c>
@@ -1881,7 +2052,7 @@
       <c r="BY17" s="13"/>
       <c r="BZ17" s="13"/>
     </row>
-    <row r="18" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>7</v>
       </c>
@@ -1955,7 +2126,7 @@
       <c r="BY18" s="19"/>
       <c r="BZ18" s="19"/>
     </row>
-    <row r="19" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>7</v>
       </c>
@@ -2029,7 +2200,7 @@
       <c r="BY19" s="13"/>
       <c r="BZ19" s="13"/>
     </row>
-    <row r="20" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>7</v>
       </c>
@@ -2103,7 +2274,7 @@
       <c r="BY20" s="13"/>
       <c r="BZ20" s="13"/>
     </row>
-    <row r="21" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
         <v>7</v>
       </c>
@@ -2177,7 +2348,7 @@
       <c r="BY21" s="13"/>
       <c r="BZ21" s="13"/>
     </row>
-    <row r="22" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>7</v>
       </c>
@@ -2251,7 +2422,7 @@
       <c r="BY22" s="13"/>
       <c r="BZ22" s="13"/>
     </row>
-    <row r="23" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>7</v>
       </c>
@@ -2325,7 +2496,7 @@
       <c r="BY23" s="19"/>
       <c r="BZ23" s="19"/>
     </row>
-    <row r="24" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>7</v>
       </c>
@@ -2399,7 +2570,7 @@
       <c r="BY24" s="19"/>
       <c r="BZ24" s="19"/>
     </row>
-    <row r="25" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>7</v>
       </c>
@@ -2473,7 +2644,7 @@
       <c r="BY25" s="13"/>
       <c r="BZ25" s="13"/>
     </row>
-    <row r="26" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>7</v>
       </c>
@@ -2547,7 +2718,7 @@
       <c r="BY26" s="13"/>
       <c r="BZ26" s="13"/>
     </row>
-    <row r="27" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
         <v>17</v>
       </c>
@@ -2612,7 +2783,7 @@
       <c r="BS27" s="24"/>
       <c r="BW27" s="24"/>
     </row>
-    <row r="28" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
         <v>17</v>
       </c>
@@ -2677,7 +2848,7 @@
       <c r="BS28" s="24"/>
       <c r="BW28" s="24"/>
     </row>
-    <row r="29" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
         <v>17</v>
       </c>
@@ -2742,7 +2913,7 @@
       <c r="BS29" s="24"/>
       <c r="BW29" s="24"/>
     </row>
-    <row r="30" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
         <v>17</v>
       </c>
@@ -2807,7 +2978,7 @@
       <c r="BS30" s="24"/>
       <c r="BW30" s="24"/>
     </row>
-    <row r="31" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
         <v>17</v>
       </c>
@@ -2872,7 +3043,7 @@
       <c r="BS31" s="24"/>
       <c r="BW31" s="24"/>
     </row>
-    <row r="32" spans="1:78" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:78" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
         <v>17</v>
       </c>
@@ -2937,7 +3108,7 @@
       <c r="BS32" s="24"/>
       <c r="BW32" s="24"/>
     </row>
-    <row r="33" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
         <v>17</v>
       </c>
@@ -3002,7 +3173,7 @@
       <c r="BS33" s="24"/>
       <c r="BW33" s="24"/>
     </row>
-    <row r="34" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
         <v>17</v>
       </c>
@@ -3067,7 +3238,7 @@
       <c r="BS34" s="24"/>
       <c r="BW34" s="24"/>
     </row>
-    <row r="35" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
         <v>17</v>
       </c>
@@ -3132,7 +3303,7 @@
       <c r="BS35" s="24"/>
       <c r="BW35" s="24"/>
     </row>
-    <row r="36" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
         <v>17</v>
       </c>
@@ -3197,7 +3368,7 @@
       <c r="BS36" s="24"/>
       <c r="BW36" s="24"/>
     </row>
-    <row r="37" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
         <v>17</v>
       </c>
@@ -3259,7 +3430,7 @@
       <c r="BQ37" s="12"/>
       <c r="BS37" s="24"/>
     </row>
-    <row r="38" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="6" t="s">
         <v>17</v>
       </c>
@@ -3321,7 +3492,7 @@
       <c r="BQ38" s="9"/>
       <c r="BS38" s="24"/>
     </row>
-    <row r="39" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="6" t="s">
         <v>17</v>
       </c>
@@ -3383,7 +3554,7 @@
       <c r="BQ39" s="18"/>
       <c r="BS39" s="24"/>
     </row>
-    <row r="40" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="6" t="s">
         <v>17</v>
       </c>
@@ -3445,7 +3616,7 @@
       <c r="BQ40" s="18"/>
       <c r="BS40" s="24"/>
     </row>
-    <row r="41" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
         <v>17</v>
       </c>
@@ -3507,7 +3678,7 @@
       <c r="BQ41" s="21"/>
       <c r="BS41" s="24"/>
     </row>
-    <row r="42" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
         <v>17</v>
       </c>
@@ -3569,7 +3740,7 @@
       <c r="BQ42" s="12"/>
       <c r="BS42" s="24"/>
     </row>
-    <row r="43" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
         <v>17</v>
       </c>
@@ -3631,7 +3802,7 @@
       <c r="BQ43" s="9"/>
       <c r="BS43" s="25"/>
     </row>
-    <row r="44" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
         <v>17</v>
       </c>
@@ -3693,7 +3864,7 @@
       <c r="BQ44" s="9"/>
       <c r="BS44" s="24"/>
     </row>
-    <row r="45" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
         <v>17</v>
       </c>
@@ -3755,7 +3926,7 @@
       <c r="BQ45" s="18"/>
       <c r="BS45" s="24"/>
     </row>
-    <row r="46" spans="1:75" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:75" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>17</v>
       </c>
@@ -3847,10 +4018,12 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4772,94 +4945,1128 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="32"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
+      <c r="A29" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D29" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E29" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24">
+        <v>651</v>
+      </c>
+      <c r="I29" s="24">
+        <v>651</v>
+      </c>
+      <c r="J29" s="24"/>
     </row>
     <row r="30" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="32"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
+      <c r="A30" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D30" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E30" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F30" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24">
+        <v>643.20000000000005</v>
+      </c>
+      <c r="I30" s="24">
+        <v>643.20000000000005</v>
+      </c>
+      <c r="J30" s="24"/>
     </row>
     <row r="31" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="32"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
+      <c r="A31" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F31" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24">
+        <v>859.8</v>
+      </c>
+      <c r="I31" s="24">
+        <v>859.8</v>
+      </c>
+      <c r="J31" s="24"/>
     </row>
     <row r="32" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="32"/>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-    </row>
-    <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="32"/>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-    </row>
-    <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="32"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-    </row>
-    <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="32"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-    </row>
-    <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="32"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-    </row>
-    <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="32"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
+      <c r="A32" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24">
+        <v>-1.2</v>
+      </c>
+      <c r="I32" s="24">
+        <v>-1.2</v>
+      </c>
+      <c r="J32" s="24"/>
+    </row>
+    <row r="33" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A33" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24">
+        <v>-2.2000000000000002</v>
+      </c>
+      <c r="I33" s="24">
+        <v>-2.2000000000000002</v>
+      </c>
+      <c r="J33" s="24"/>
+    </row>
+    <row r="34" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A34" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F34" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24">
+        <v>6.2</v>
+      </c>
+      <c r="I34" s="24">
+        <v>6.2</v>
+      </c>
+      <c r="J34" s="24"/>
+    </row>
+    <row r="35" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E35" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24">
+        <v>911.3</v>
+      </c>
+      <c r="I35" s="24">
+        <v>911.3</v>
+      </c>
+      <c r="J35" s="24">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A36" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D36" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E36" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F36" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24">
+        <v>852.2</v>
+      </c>
+      <c r="I36" s="24">
+        <v>852.2</v>
+      </c>
+      <c r="J36" s="24">
+        <v>643.20000000000005</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A37" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E37" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F37" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="G37" s="24"/>
+      <c r="H37" s="24">
+        <v>1259.5</v>
+      </c>
+      <c r="I37" s="24">
+        <v>1259.5</v>
+      </c>
+      <c r="J37" s="24">
+        <v>859.8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A38" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E38" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G38" s="24"/>
+      <c r="H38" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="I38" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="J38" s="24">
+        <v>-1.2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A39" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D39" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E39" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F39" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="I39" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="J39" s="24">
+        <v>-2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A40" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B40" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E40" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F40" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="I40" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="J40" s="24">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A41" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C41" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D41" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E41" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="G41" s="24"/>
+      <c r="H41" s="24">
+        <v>897.7</v>
+      </c>
+      <c r="I41" s="24">
+        <v>897.7</v>
+      </c>
+      <c r="J41" s="24">
+        <v>911.3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A42" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D42" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E42" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F42" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G42" s="24"/>
+      <c r="H42" s="24">
+        <v>953.5</v>
+      </c>
+      <c r="I42" s="24">
+        <v>953.5</v>
+      </c>
+      <c r="J42" s="24">
+        <v>852.2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A43" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D43" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E43" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="G43" s="24"/>
+      <c r="H43" s="24">
+        <v>1142.5</v>
+      </c>
+      <c r="I43" s="24">
+        <v>1142.5</v>
+      </c>
+      <c r="J43" s="24">
+        <v>1259.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A44" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C44" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D44" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E44" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F44" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G44" s="24"/>
+      <c r="H44" s="24">
+        <v>-0.8</v>
+      </c>
+      <c r="I44" s="24">
+        <v>-0.8</v>
+      </c>
+      <c r="J44" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A45" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C45" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E45" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F45" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G45" s="24"/>
+      <c r="H45" s="24">
+        <v>-4.8</v>
+      </c>
+      <c r="I45" s="24">
+        <v>-4.8</v>
+      </c>
+      <c r="J45" s="24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A46" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C46" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D46" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E46" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F46" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G46" s="24"/>
+      <c r="H46" s="24">
+        <v>4.8</v>
+      </c>
+      <c r="I46" s="24">
+        <v>4.8</v>
+      </c>
+      <c r="J46" s="24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A47" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C47" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D47" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E47" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F47" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="G47" s="24"/>
+      <c r="H47" s="24">
+        <v>823.2</v>
+      </c>
+      <c r="I47" s="24">
+        <v>823.2</v>
+      </c>
+      <c r="J47" s="24">
+        <v>897.7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A48" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C48" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D48" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E48" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F48" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G48" s="24"/>
+      <c r="H48" s="24">
+        <v>876.5</v>
+      </c>
+      <c r="I48" s="24">
+        <v>876.5</v>
+      </c>
+      <c r="J48" s="24">
+        <v>953.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A49" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C49" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D49" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E49" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F49" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="G49" s="24"/>
+      <c r="H49" s="24">
+        <v>1020.5</v>
+      </c>
+      <c r="I49" s="24">
+        <v>1020.5</v>
+      </c>
+      <c r="J49" s="24">
+        <v>1142.5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A50" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C50" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D50" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E50" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F50" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G50" s="24"/>
+      <c r="H50" s="24">
+        <v>0.8</v>
+      </c>
+      <c r="I50" s="24">
+        <v>0.8</v>
+      </c>
+      <c r="J50" s="24">
+        <v>-0.8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A51" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B51" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C51" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D51" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E51" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F51" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G51" s="24"/>
+      <c r="H51" s="24">
+        <v>-3.2</v>
+      </c>
+      <c r="I51" s="24">
+        <v>-3.2</v>
+      </c>
+      <c r="J51" s="24">
+        <v>-4.8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A52" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="D52" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E52" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F52" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G52" s="24"/>
+      <c r="H52" s="24">
+        <v>4</v>
+      </c>
+      <c r="I52" s="24">
+        <v>4</v>
+      </c>
+      <c r="J52" s="24">
+        <v>4.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EACB0132-BF50-F94C-A1BF-4428E785A278}">
+  <dimension ref="A1:AB7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="4.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="K1" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="L1" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="M1" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
+      <c r="AB1" s="24"/>
+    </row>
+    <row r="2" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="15">
+        <v>0.2</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="15">
+        <v>1</v>
+      </c>
+      <c r="G2" s="15">
+        <v>20</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L2" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="M2" s="15">
+        <v>201906</v>
+      </c>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="V2" s="24"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="24"/>
+      <c r="Z2" s="24"/>
+      <c r="AA2" s="24"/>
+      <c r="AB2" s="24"/>
+    </row>
+    <row r="3" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D3" s="15">
+        <v>0.45</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="15">
+        <v>1</v>
+      </c>
+      <c r="G3" s="15">
+        <v>4</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="M3" s="15">
+        <v>201906</v>
+      </c>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="24"/>
+      <c r="X3" s="24"/>
+      <c r="Y3" s="24"/>
+      <c r="Z3" s="24"/>
+      <c r="AA3" s="24"/>
+      <c r="AB3" s="24"/>
+    </row>
+    <row r="4" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="15">
+        <v>0.75</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="15">
+        <v>1</v>
+      </c>
+      <c r="G4" s="15">
+        <v>1</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="M4" s="15">
+        <v>201906</v>
+      </c>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+      <c r="W4" s="24"/>
+      <c r="X4" s="24"/>
+      <c r="Y4" s="24"/>
+      <c r="Z4" s="24"/>
+      <c r="AA4" s="24"/>
+      <c r="AB4" s="24"/>
+    </row>
+    <row r="5" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="15">
+        <v>0.95</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="15">
+        <v>1</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L5" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="M5" s="15">
+        <v>201906</v>
+      </c>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
+      <c r="V5" s="24"/>
+      <c r="W5" s="24"/>
+      <c r="X5" s="24"/>
+      <c r="Y5" s="24"/>
+      <c r="Z5" s="24"/>
+      <c r="AA5" s="24"/>
+      <c r="AB5" s="24"/>
+    </row>
+    <row r="6" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="15">
+        <v>1.45</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="F6" s="15">
+        <v>1.518</v>
+      </c>
+      <c r="G6" s="15">
+        <v>0.13</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L6" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="M6" s="15">
+        <v>201808</v>
+      </c>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="24"/>
+      <c r="S6" s="24"/>
+      <c r="T6" s="24"/>
+      <c r="U6" s="24"/>
+      <c r="V6" s="24"/>
+      <c r="W6" s="24"/>
+      <c r="X6" s="24"/>
+      <c r="Y6" s="24"/>
+      <c r="Z6" s="24"/>
+      <c r="AA6" s="24"/>
+    </row>
+    <row r="7" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="15">
+        <v>1.4</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" s="15">
+        <v>1.518</v>
+      </c>
+      <c r="G7" s="15">
+        <v>0.13</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L7" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="M7" s="15">
+        <v>202007</v>
+      </c>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="24"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24"/>
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
+      <c r="V7" s="24"/>
+      <c r="W7" s="24"/>
+      <c r="X7" s="24"/>
+      <c r="Y7" s="24"/>
+      <c r="Z7" s="24"/>
+      <c r="AA7" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Link objectives in PSF & show their information
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F08F61-A961-E24A-8D60-D986712F5C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA29E77-2C43-2547-9558-5ECFB1C0DE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="93">
   <si>
     <t>Site</t>
   </si>
@@ -4018,7 +4018,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
@@ -5649,6 +5649,96 @@
         <v>4</v>
       </c>
       <c r="J52" s="24">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A53" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B53" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C53" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E53" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F53" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G53" s="24"/>
+      <c r="H53" s="24">
+        <v>0.8</v>
+      </c>
+      <c r="I53" s="24">
+        <v>0.8</v>
+      </c>
+      <c r="J53" s="24">
+        <v>-0.8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A54" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B54" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C54" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E54" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F54" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G54" s="24"/>
+      <c r="H54" s="24">
+        <v>-3.2</v>
+      </c>
+      <c r="I54" s="24">
+        <v>-3.2</v>
+      </c>
+      <c r="J54" s="24">
+        <v>-4.8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A55" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D55" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E55" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F55" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G55" s="24"/>
+      <c r="H55" s="24">
+        <v>4</v>
+      </c>
+      <c r="I55" s="24">
+        <v>4</v>
+      </c>
+      <c r="J55" s="24">
         <v>4.8</v>
       </c>
     </row>
@@ -6070,5 +6160,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Make PSF - objective ID selections: 'mag/na (ID)'
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA29E77-2C43-2547-9558-5ECFB1C0DE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8AD5F31-F6E7-E74A-9C40-52D09EF6228C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="94">
   <si>
     <t>Site</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>cupboard</t>
+  </si>
+  <si>
+    <t>ID999</t>
   </si>
 </sst>
 </file>
@@ -5720,7 +5723,7 @@
         <v>20</v>
       </c>
       <c r="C55" s="24" t="s">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="D55" s="24" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
Add Field distortion/uniformity place-holder
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8AD5F31-F6E7-E74A-9C40-52D09EF6228C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F875AEA-5385-8B45-B3F0-49354131C50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="laser_power_measurements" sheetId="1" r:id="rId1"/>
     <sheet name="psf_measurements" sheetId="2" r:id="rId2"/>
-    <sheet name="objective_db" sheetId="3" r:id="rId3"/>
+    <sheet name="field_dist_uni" sheetId="4" r:id="rId3"/>
+    <sheet name="objective_db" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="98">
   <si>
     <t>Site</t>
   </si>
@@ -317,6 +318,18 @@
   </si>
   <si>
     <t>ID999</t>
+  </si>
+  <si>
+    <t>Leica DMi8</t>
+  </si>
+  <si>
+    <t>63x/1.4</t>
+  </si>
+  <si>
+    <t>Test omero ID</t>
+  </si>
+  <si>
+    <t>omero3021627</t>
   </si>
 </sst>
 </file>
@@ -461,7 +474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -537,6 +550,7 @@
     </xf>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5752,6 +5766,57 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF13278A-16E7-1B4C-AB14-E4151DDE9509}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="35" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="35" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="35">
+        <v>20260309</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A2" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EACB0132-BF50-F94C-A1BF-4428E785A278}">
   <dimension ref="A1:AB7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>

</xml_diff>

<commit_message>
Add distortion/uniformity upload, & make empty spreadsheet possible
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F875AEA-5385-8B45-B3F0-49354131C50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33E11F9A-053D-C649-9DD9-8E7F3D3EDC54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="98">
   <si>
     <t>Site</t>
   </si>
@@ -5767,17 +5767,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF13278A-16E7-1B4C-AB14-E4151DDE9509}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="35" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:6" s="35" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
@@ -5790,11 +5791,14 @@
       <c r="D1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="35">
+      <c r="E1" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="35">
         <v>20260309</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A2" s="24" t="s">
         <v>17</v>
       </c>
@@ -5808,6 +5812,9 @@
         <v>96</v>
       </c>
       <c r="E2" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FieldData class and start distortion app
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33E11F9A-053D-C649-9DD9-8E7F3D3EDC54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771D5799-B8EB-0F49-822A-31C01DB0B9F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="laser_power_measurements" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="107">
   <si>
     <t>Site</t>
   </si>
@@ -248,88 +248,115 @@
     <t>MRD00045</t>
   </si>
   <si>
+    <t>10x</t>
+  </si>
+  <si>
+    <t>MRD00105</t>
+  </si>
+  <si>
+    <t>20x</t>
+  </si>
+  <si>
+    <t>MRD00205</t>
+  </si>
+  <si>
+    <t>40x</t>
+  </si>
+  <si>
+    <t>0.25-0-17</t>
+  </si>
+  <si>
+    <t>MRD00405</t>
+  </si>
+  <si>
+    <t>ID5</t>
+  </si>
+  <si>
+    <t>100x</t>
+  </si>
+  <si>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>EXT Ph4</t>
+  </si>
+  <si>
+    <t>Ti2</t>
+  </si>
+  <si>
+    <t>MRD01905</t>
+  </si>
+  <si>
+    <t>ID19</t>
+  </si>
+  <si>
+    <t>60x</t>
+  </si>
+  <si>
+    <t>EXT Ph3</t>
+  </si>
+  <si>
+    <t>Cupboard</t>
+  </si>
+  <si>
+    <t>CSU-W1</t>
+  </si>
+  <si>
+    <t>MRD01605</t>
+  </si>
+  <si>
+    <t>cupboard</t>
+  </si>
+  <si>
+    <t>ID999</t>
+  </si>
+  <si>
+    <t>Test_microscope</t>
+  </si>
+  <si>
+    <t>Test_63x</t>
+  </si>
+  <si>
+    <t>Test_info</t>
+  </si>
+  <si>
+    <t>omero3454869_ch-1</t>
+  </si>
+  <si>
+    <t>omero3454869_ch-2</t>
+  </si>
+  <si>
+    <t>Alexa 647</t>
+  </si>
+  <si>
+    <t>omero3454869_ch-3</t>
+  </si>
+  <si>
+    <t>omero3454869_ch-0</t>
+  </si>
+  <si>
+    <t>IDN5</t>
+  </si>
+  <si>
+    <t>IDN4</t>
+  </si>
+  <si>
+    <t>IDN1</t>
+  </si>
+  <si>
+    <t>IDN2</t>
+  </si>
+  <si>
+    <t>IDN3</t>
+  </si>
+  <si>
     <t>ID2</t>
   </si>
   <si>
-    <t>10x</t>
-  </si>
-  <si>
-    <t>MRD00105</t>
-  </si>
-  <si>
     <t>ID3</t>
   </si>
   <si>
-    <t>20x</t>
-  </si>
-  <si>
-    <t>MRD00205</t>
-  </si>
-  <si>
     <t>ID4</t>
-  </si>
-  <si>
-    <t>40x</t>
-  </si>
-  <si>
-    <t>0.25-0-17</t>
-  </si>
-  <si>
-    <t>MRD00405</t>
-  </si>
-  <si>
-    <t>ID5</t>
-  </si>
-  <si>
-    <t>100x</t>
-  </si>
-  <si>
-    <t>Oil</t>
-  </si>
-  <si>
-    <t>EXT Ph4</t>
-  </si>
-  <si>
-    <t>Ti2</t>
-  </si>
-  <si>
-    <t>MRD01905</t>
-  </si>
-  <si>
-    <t>ID19</t>
-  </si>
-  <si>
-    <t>60x</t>
-  </si>
-  <si>
-    <t>EXT Ph3</t>
-  </si>
-  <si>
-    <t>Cupboard</t>
-  </si>
-  <si>
-    <t>CSU-W1</t>
-  </si>
-  <si>
-    <t>MRD01605</t>
-  </si>
-  <si>
-    <t>cupboard</t>
-  </si>
-  <si>
-    <t>ID999</t>
-  </si>
-  <si>
-    <t>Leica DMi8</t>
-  </si>
-  <si>
-    <t>63x/1.4</t>
-  </si>
-  <si>
-    <t>Test omero ID</t>
-  </si>
-  <si>
-    <t>omero3021627</t>
   </si>
 </sst>
 </file>
@@ -4969,7 +4996,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D29" s="24" t="s">
         <v>41</v>
@@ -4997,7 +5024,7 @@
         <v>20</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D30" s="24" t="s">
         <v>41</v>
@@ -5025,7 +5052,7 @@
         <v>20</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D31" s="24" t="s">
         <v>41</v>
@@ -5053,7 +5080,7 @@
         <v>20</v>
       </c>
       <c r="C32" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D32" s="24" t="s">
         <v>41</v>
@@ -5081,7 +5108,7 @@
         <v>20</v>
       </c>
       <c r="C33" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D33" s="24" t="s">
         <v>41</v>
@@ -5109,7 +5136,7 @@
         <v>20</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D34" s="24" t="s">
         <v>41</v>
@@ -5137,7 +5164,7 @@
         <v>20</v>
       </c>
       <c r="C35" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D35" s="24" t="s">
         <v>41</v>
@@ -5167,7 +5194,7 @@
         <v>20</v>
       </c>
       <c r="C36" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D36" s="24" t="s">
         <v>41</v>
@@ -5197,7 +5224,7 @@
         <v>20</v>
       </c>
       <c r="C37" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D37" s="24" t="s">
         <v>41</v>
@@ -5227,7 +5254,7 @@
         <v>20</v>
       </c>
       <c r="C38" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D38" s="24" t="s">
         <v>41</v>
@@ -5257,7 +5284,7 @@
         <v>20</v>
       </c>
       <c r="C39" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D39" s="24" t="s">
         <v>41</v>
@@ -5287,7 +5314,7 @@
         <v>20</v>
       </c>
       <c r="C40" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D40" s="24" t="s">
         <v>41</v>
@@ -5317,7 +5344,7 @@
         <v>20</v>
       </c>
       <c r="C41" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D41" s="24" t="s">
         <v>41</v>
@@ -5347,7 +5374,7 @@
         <v>20</v>
       </c>
       <c r="C42" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D42" s="24" t="s">
         <v>41</v>
@@ -5377,7 +5404,7 @@
         <v>20</v>
       </c>
       <c r="C43" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D43" s="24" t="s">
         <v>41</v>
@@ -5407,7 +5434,7 @@
         <v>20</v>
       </c>
       <c r="C44" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D44" s="24" t="s">
         <v>41</v>
@@ -5437,7 +5464,7 @@
         <v>20</v>
       </c>
       <c r="C45" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D45" s="24" t="s">
         <v>41</v>
@@ -5467,7 +5494,7 @@
         <v>20</v>
       </c>
       <c r="C46" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D46" s="24" t="s">
         <v>41</v>
@@ -5497,7 +5524,7 @@
         <v>20</v>
       </c>
       <c r="C47" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D47" s="24" t="s">
         <v>41</v>
@@ -5527,7 +5554,7 @@
         <v>20</v>
       </c>
       <c r="C48" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D48" s="24" t="s">
         <v>41</v>
@@ -5557,7 +5584,7 @@
         <v>20</v>
       </c>
       <c r="C49" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D49" s="24" t="s">
         <v>41</v>
@@ -5587,7 +5614,7 @@
         <v>20</v>
       </c>
       <c r="C50" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D50" s="24" t="s">
         <v>41</v>
@@ -5617,7 +5644,7 @@
         <v>20</v>
       </c>
       <c r="C51" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D51" s="24" t="s">
         <v>41</v>
@@ -5647,7 +5674,7 @@
         <v>20</v>
       </c>
       <c r="C52" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D52" s="24" t="s">
         <v>41</v>
@@ -5737,7 +5764,7 @@
         <v>20</v>
       </c>
       <c r="C55" s="24" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D55" s="24" t="s">
         <v>41</v>
@@ -5767,7 +5794,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF13278A-16E7-1B4C-AB14-E4151DDE9509}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -5794,8 +5821,8 @@
       <c r="E1" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="35">
-        <v>20260309</v>
+      <c r="F1" s="24">
+        <v>20260101</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.15">
@@ -5803,19 +5830,79 @@
         <v>17</v>
       </c>
       <c r="B2" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" s="24">
+        <v>488</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="24" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A3" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" s="24">
+        <v>561</v>
+      </c>
+      <c r="F3" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="D2" s="24" t="s">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A4" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="F4" s="24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A5" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>97</v>
+      <c r="F5" s="24" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -5825,10 +5912,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EACB0132-BF50-F94C-A1BF-4428E785A278}">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="4.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -5957,13 +6044,13 @@
     </row>
     <row r="3" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>62</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D3" s="15">
         <v>0.45</v>
@@ -5990,7 +6077,7 @@
         <v>68</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M3" s="15">
         <v>201906</v>
@@ -6013,13 +6100,13 @@
     </row>
     <row r="4" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>73</v>
+        <v>105</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>62</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D4" s="15">
         <v>0.75</v>
@@ -6046,7 +6133,7 @@
         <v>68</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M4" s="15">
         <v>201906</v>
@@ -6069,13 +6156,13 @@
     </row>
     <row r="5" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>62</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D5" s="15">
         <v>0.95</v>
@@ -6087,7 +6174,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>65</v>
@@ -6102,7 +6189,7 @@
         <v>68</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="M5" s="15">
         <v>201906</v>
@@ -6125,19 +6212,19 @@
     </row>
     <row r="6" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>62</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D6" s="15">
         <v>1.45</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F6" s="15">
         <v>1.518</v>
@@ -6146,19 +6233,19 @@
         <v>0.13</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="K6" s="15" t="s">
         <v>68</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="M6" s="15">
         <v>201808</v>
@@ -6180,19 +6267,19 @@
     </row>
     <row r="7" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>62</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D7" s="15">
         <v>1.4</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F7" s="15">
         <v>1.518</v>
@@ -6201,19 +6288,19 @@
         <v>0.13</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="K7" s="15" t="s">
         <v>68</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="M7" s="15">
         <v>202007</v>
@@ -6233,7 +6320,213 @@
       <c r="Z7" s="24"/>
       <c r="AA7" s="24"/>
     </row>
+    <row r="8" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="15">
+        <v>0.2</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="15">
+        <v>1</v>
+      </c>
+      <c r="G8" s="15">
+        <v>20</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L8" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="M8" s="15">
+        <v>201906</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="15">
+        <v>0.45</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="15">
+        <v>1</v>
+      </c>
+      <c r="G9" s="15">
+        <v>4</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L9" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="M9" s="15">
+        <v>201906</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="15">
+        <v>0.75</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="15">
+        <v>1</v>
+      </c>
+      <c r="G10" s="15">
+        <v>1</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J10" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L10" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="M10" s="15">
+        <v>201906</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="15">
+        <v>0.95</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" s="15">
+        <v>1</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J11" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L11" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="M11" s="15">
+        <v>201906</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="15">
+        <v>1.45</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="15">
+        <v>1.518</v>
+      </c>
+      <c r="G12" s="15">
+        <v>0.13</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="J12" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="K12" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="L12" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="M12" s="15">
+        <v>201808</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Add distortion plots for channels
</commit_message>
<xml_diff>
--- a/example_files/metroloshiny_data_example.xlsx
+++ b/example_files/metroloshiny_data_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/loic/Documents/Coding_projects/metroloshiny/example_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771D5799-B8EB-0F49-822A-31C01DB0B9F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF21AC18-C359-A848-9794-C340A35821F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29600" windowHeight="21620" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29320" yWindow="10860" windowWidth="29620" windowHeight="21640" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="laser_power_measurements" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="109">
   <si>
     <t>Site</t>
   </si>
@@ -357,6 +357,12 @@
   </si>
   <si>
     <t>ID4</t>
+  </si>
+  <si>
+    <t>Test_microscope2</t>
+  </si>
+  <si>
+    <t>noID</t>
   </si>
 </sst>
 </file>
@@ -5794,18 +5800,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF13278A-16E7-1B4C-AB14-E4151DDE9509}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="35" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
@@ -5824,8 +5830,17 @@
       <c r="F1" s="24">
         <v>20260101</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="G1" s="24">
+        <v>20260109</v>
+      </c>
+      <c r="H1" s="24">
+        <v>20260120</v>
+      </c>
+      <c r="I1" s="24">
+        <v>20260104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A2" s="24" t="s">
         <v>17</v>
       </c>
@@ -5844,8 +5859,15 @@
       <c r="F2" s="24" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="G2" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="H2" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" s="24"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A3" s="24" t="s">
         <v>17</v>
       </c>
@@ -5864,8 +5886,15 @@
       <c r="F3" s="24" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="G3" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="H3" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="I3" s="24"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A4" s="24" t="s">
         <v>17</v>
       </c>
@@ -5884,8 +5913,15 @@
       <c r="F4" s="24" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="G4" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="H4" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="I4" s="24"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A5" s="24" t="s">
         <v>17</v>
       </c>
@@ -5904,9 +5940,118 @@
       <c r="F5" s="24" t="s">
         <v>98</v>
       </c>
+      <c r="G5" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A6" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="24">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A7" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E7" s="24">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A8" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A9" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A10" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A11" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>